<commit_message>
SUC scan works well. AACCUP Program scan needs tweaking
</commit_message>
<xml_diff>
--- a/context/copctemplate.xlsx
+++ b/context/copctemplate.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Quality-Assurance-System\context\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715F7DC9-06D4-4DAD-9B57-1EE10B4C5035}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="10965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,265 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="84">
+  <si>
+    <t>I. Profile</t>
+  </si>
+  <si>
+    <t>Name of Program: Bachelor of Early Childhood Education</t>
+  </si>
+  <si>
+    <t>Majors: None</t>
+  </si>
+  <si>
+    <t>Program Pathway</t>
+  </si>
+  <si>
+    <t>History</t>
+  </si>
+  <si>
+    <t>Graduate Profile</t>
+  </si>
+  <si>
+    <t>COPC</t>
+  </si>
+  <si>
+    <t>II. School Administrators</t>
+  </si>
+  <si>
+    <t>Organizational Structure</t>
+  </si>
+  <si>
+    <t>President</t>
+  </si>
+  <si>
+    <t>Vice-President for Academic Affairs</t>
+  </si>
+  <si>
+    <t>Vice-President for Administration and Finance</t>
+  </si>
+  <si>
+    <t>Directors</t>
+  </si>
+  <si>
+    <t>Dean/Program Head</t>
+  </si>
+  <si>
+    <t>III. Faculty Members</t>
+  </si>
+  <si>
+    <t>List General Education Faculty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of Professional Education Faculty </t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of Specialization Faculty </t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of Full Time Faculty </t>
+  </si>
+  <si>
+    <t>List of Part-time Faculty</t>
+  </si>
+  <si>
+    <t>IV. Non-Teaching Personnel</t>
+  </si>
+  <si>
+    <t>College Registrar</t>
+  </si>
+  <si>
+    <t>College Guidance Counselor</t>
+  </si>
+  <si>
+    <t>Administrative Staff</t>
+  </si>
+  <si>
+    <t>V. Curriculum</t>
+  </si>
+  <si>
+    <t>CMO</t>
+  </si>
+  <si>
+    <t>Complete set of Program Outcomes, including its proposed additional program outcomes</t>
+  </si>
+  <si>
+    <t>Performance indicators for each outcome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level of attainment of each indicator </t>
+  </si>
+  <si>
+    <t>Distribution of subjects per term</t>
+  </si>
+  <si>
+    <t>Summary of units It shall depend on the reviewed prospectus</t>
+  </si>
+  <si>
+    <t>Course Description (by subject) It shall depend on the reviewed prospectus</t>
+  </si>
+  <si>
+    <t>Outcomes-based syllabus (by subject)</t>
+  </si>
+  <si>
+    <t>System of program assessment and evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System of Program Continuous Quality Improvement (CQI) </t>
+  </si>
+  <si>
+    <t>VI. Library</t>
+  </si>
+  <si>
+    <t>Librarian</t>
+  </si>
+  <si>
+    <t>Transcript of Records</t>
+  </si>
+  <si>
+    <t>Appointment</t>
+  </si>
+  <si>
+    <t>Professional License</t>
+  </si>
+  <si>
+    <t>Facilities</t>
+  </si>
+  <si>
+    <t>Floor space in sq. m.</t>
+  </si>
+  <si>
+    <t>Pictures</t>
+  </si>
+  <si>
+    <t>Seating Capacity</t>
+  </si>
+  <si>
+    <t>Combined Number of students and faculty at one time</t>
+  </si>
+  <si>
+    <t>Library Collections</t>
+  </si>
+  <si>
+    <t>List of 5 non-duplicated book titles per subject in the curriculum published within the last five years</t>
+  </si>
+  <si>
+    <t>List of book collections/ accessioned books</t>
+  </si>
+  <si>
+    <t>Start- up 3,000 library collections (for initial permit) Minimum of 5,000 library Collections (for recognition)</t>
+  </si>
+  <si>
+    <t>List of subscriptions to relevant professional journals (Note: List should be in spreadsheet to include author, title of book, year of publication and number of volumes)</t>
+  </si>
+  <si>
+    <t>Active subscription to at least 4 refereed journals and periodicals in education that are published locally and internationally.</t>
+  </si>
+  <si>
+    <t>VII. Physical Facilities</t>
+  </si>
+  <si>
+    <t>Document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIII. List of Equipment and other Instructional Devices/Aids </t>
+  </si>
+  <si>
+    <t>List</t>
+  </si>
+  <si>
+    <t>IX. Support Facilities</t>
+  </si>
+  <si>
+    <t>Audio Visual Room</t>
+  </si>
+  <si>
+    <t>Sports and recreational, if outsourced to include notarized MOA</t>
+  </si>
+  <si>
+    <t>Canteen</t>
+  </si>
+  <si>
+    <t>Faculty Lounge</t>
+  </si>
+  <si>
+    <t>Student Lounge</t>
+  </si>
+  <si>
+    <t>(2) Science Laboratories (for 3 ITE Programs)</t>
+  </si>
+  <si>
+    <t>ECE Hub</t>
+  </si>
+  <si>
+    <t>Simulation/Demo Room (for 3 ITE Programs)</t>
+  </si>
+  <si>
+    <t>X. Support Services</t>
+  </si>
+  <si>
+    <t>Guidance and Counselling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical and Dental Services for students and Faculty, if outsourced to include notarized MOA </t>
+  </si>
+  <si>
+    <t>XI. NSTP</t>
+  </si>
+  <si>
+    <t>Coordinator's Profile</t>
+  </si>
+  <si>
+    <t>Appoinment</t>
+  </si>
+  <si>
+    <t>NSTP Office</t>
+  </si>
+  <si>
+    <t>Affiliation to Accredited NSTP Provider, if outsourced to include notarized MOA</t>
+  </si>
+  <si>
+    <t>XII. Admission and Retention</t>
+  </si>
+  <si>
+    <t>A. The institution must have in place a selective admission policy for TE programs. This policy shall include passing an admission examination. TEIs may use either of the following admission examinations:</t>
+  </si>
+  <si>
+    <t>a. An admission exam developed and validated by the TEI;</t>
+  </si>
+  <si>
+    <t>b. An admission exam developed and validated by another TEI and used by TEI under a consortium agreement;</t>
+  </si>
+  <si>
+    <t>c. An admission exam developed and validated by private testing centers and used by TEI for a fee;</t>
+  </si>
+  <si>
+    <t>d. Some other standardized tests for teaching aptitude; or</t>
+  </si>
+  <si>
+    <t>e. Some other national qualifications examinations which may be developed in the future.</t>
+  </si>
+  <si>
+    <t>XIII. Research Projects</t>
+  </si>
+  <si>
+    <t>Accomplishment Reports</t>
+  </si>
+  <si>
+    <t>XIV. Extension Projects</t>
+  </si>
+  <si>
+    <t>XV. Internationalization</t>
+  </si>
+  <si>
+    <t>XVI. Best Practices</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -330,10 +593,420 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A3:B92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>51</v>
+      </c>
+      <c r="B57" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>53</v>
+      </c>
+      <c r="B59" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>55</v>
+      </c>
+      <c r="B61" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>64</v>
+      </c>
+      <c r="B70" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>67</v>
+      </c>
+      <c r="B73" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>72</v>
+      </c>
+      <c r="B79" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>79</v>
+      </c>
+      <c r="B86" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>81</v>
+      </c>
+      <c r="B88" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>82</v>
+      </c>
+      <c r="B90" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>83</v>
+      </c>
+      <c r="B92" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>